<commit_message>
Fix #19822 - [Featutr] Update Citeo Export (FR)
</commit_message>
<xml_diff>
--- a/becpg-plm/becpg-plm-core/src/main/resources/beCPG/birt/exportsearch/product/fr/ExportCiteo.xlsx
+++ b/becpg-plm/becpg-plm-core/src/main/resources/beCPG/birt/exportsearch/product/fr/ExportCiteo.xlsx
@@ -5,14 +5,14 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Eco emballage (Citeo 2023)" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="Eco emballage" sheetId="1" state="visible" r:id="rId2"/>
     <sheet name="Matériaux" sheetId="2" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Matériaux!$B$3:$H$4</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Matériaux!$B$3:$H$3</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -77,7 +77,7 @@
     <t xml:space="preserve">gs1:packUnitNumber</t>
   </si>
   <si>
-    <t xml:space="preserve">ljs:packUnitNumberLight</t>
+    <t xml:space="preserve">formula|""</t>
   </si>
   <si>
     <t xml:space="preserve">excel|IFERROR(IF(G2="","",VLOOKUP(E2&amp;"C"&amp;INDIRECT("K"&amp;ROW($A$2)+5)&amp;"P",Matériaux!$F$4:$G$10000,2,FALSE)),"")</t>
@@ -453,7 +453,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -478,6 +478,13 @@
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF2A00FF"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -806,7 +813,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="38">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -819,79 +826,79 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="true"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="true"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="true"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="true"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="true"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="true"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="true"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="true"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="true"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="true"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="true"/>
-    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="true"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="true"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="true"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="true"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="true"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="true"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="true"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="true"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="true"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="true"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="8" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="true"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="true"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="true"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -899,43 +906,47 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="9" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="8" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="9" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="9" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="9" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="10" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="10" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="11" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="11" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="12" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="12" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="13" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="13" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="13" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="13" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="true"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="8" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="8" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="14" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="14" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="14" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="12" fillId="14" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -943,11 +954,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="15" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="15" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="15" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="13" fillId="15" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -982,7 +997,7 @@
       <rgbColor rgb="FFFFFFFF"/>
       <rgbColor rgb="FFFF0000"/>
       <rgbColor rgb="FF00FF00"/>
-      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF2A00FF"/>
       <rgbColor rgb="FFFFFF00"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FF00FFFF"/>
@@ -1049,7 +1064,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AMJ7"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.7421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="0" width="11.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17.28"/>
@@ -1082,7 +1097,7 @@
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
     </row>
-    <row r="2" customFormat="false" ht="24.25" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="27.75" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -1110,7 +1125,7 @@
       <c r="I2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="J2" s="3" t="s">
         <v>11</v>
       </c>
       <c r="K2" s="2" t="s">
@@ -1183,69 +1198,69 @@
       <c r="AH2" s="1"/>
       <c r="AI2" s="2"/>
     </row>
-    <row r="3" s="3" customFormat="true" ht="22.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+    <row r="3" s="4" customFormat="true" ht="22.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4"/>
-      <c r="K3" s="5" t="s">
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="L3" s="5"/>
-      <c r="M3" s="5"/>
-      <c r="N3" s="5"/>
-      <c r="O3" s="5"/>
-      <c r="P3" s="5"/>
-      <c r="Q3" s="5"/>
-      <c r="R3" s="5"/>
-      <c r="S3" s="5"/>
-      <c r="T3" s="5"/>
-      <c r="U3" s="5"/>
-      <c r="V3" s="5"/>
-      <c r="W3" s="5"/>
-      <c r="X3" s="5"/>
-      <c r="Y3" s="5"/>
-      <c r="Z3" s="5"/>
-      <c r="AA3" s="5"/>
-      <c r="AB3" s="5"/>
-      <c r="AC3" s="5"/>
-      <c r="AD3" s="5"/>
-      <c r="AE3" s="5"/>
-      <c r="AF3" s="6" t="s">
+      <c r="L3" s="6"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="6"/>
+      <c r="O3" s="6"/>
+      <c r="P3" s="6"/>
+      <c r="Q3" s="6"/>
+      <c r="R3" s="6"/>
+      <c r="S3" s="6"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+      <c r="X3" s="6"/>
+      <c r="Y3" s="6"/>
+      <c r="Z3" s="6"/>
+      <c r="AA3" s="6"/>
+      <c r="AB3" s="6"/>
+      <c r="AC3" s="6"/>
+      <c r="AD3" s="6"/>
+      <c r="AE3" s="6"/>
+      <c r="AF3" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="AG3" s="7" t="s">
+      <c r="AG3" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="AH3" s="7"/>
-      <c r="AI3" s="8" t="s">
+      <c r="AH3" s="8"/>
+      <c r="AI3" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="AJ3" s="8"/>
-      <c r="AK3" s="9" t="s">
+      <c r="AJ3" s="9"/>
+      <c r="AK3" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="AL3" s="9"/>
-      <c r="AM3" s="9"/>
-      <c r="AN3" s="10" t="s">
+      <c r="AL3" s="10"/>
+      <c r="AM3" s="10"/>
+      <c r="AN3" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="AO3" s="11" t="s">
+      <c r="AO3" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="AP3" s="11"/>
-      <c r="AQ3" s="11"/>
-      <c r="AR3" s="11" t="n">
+      <c r="AP3" s="12"/>
+      <c r="AQ3" s="12"/>
+      <c r="AR3" s="12" t="n">
         <v>0</v>
       </c>
       <c r="AMG3" s="0"/>
@@ -1253,255 +1268,255 @@
       <c r="AMI3" s="0"/>
       <c r="AMJ3" s="0"/>
     </row>
-    <row r="4" s="16" customFormat="true" ht="22.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+    <row r="4" s="17" customFormat="true" ht="22.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="12"/>
-      <c r="L4" s="13"/>
-      <c r="M4" s="13"/>
-      <c r="N4" s="13"/>
-      <c r="O4" s="13"/>
-      <c r="P4" s="14" t="s">
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="13"/>
+      <c r="L4" s="14"/>
+      <c r="M4" s="14"/>
+      <c r="N4" s="14"/>
+      <c r="O4" s="14"/>
+      <c r="P4" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="Q4" s="14"/>
-      <c r="R4" s="14"/>
-      <c r="S4" s="14"/>
-      <c r="T4" s="14"/>
-      <c r="U4" s="14"/>
-      <c r="V4" s="14"/>
-      <c r="W4" s="14"/>
-      <c r="X4" s="14"/>
-      <c r="Y4" s="14"/>
-      <c r="Z4" s="14"/>
-      <c r="AA4" s="14"/>
-      <c r="AB4" s="14"/>
-      <c r="AC4" s="13"/>
-      <c r="AD4" s="13"/>
-      <c r="AE4" s="15"/>
-      <c r="AF4" s="6"/>
-      <c r="AG4" s="7"/>
-      <c r="AH4" s="7"/>
-      <c r="AI4" s="8"/>
-      <c r="AJ4" s="8"/>
-      <c r="AK4" s="9"/>
-      <c r="AL4" s="9"/>
-      <c r="AM4" s="9"/>
-      <c r="AN4" s="10"/>
-      <c r="AO4" s="11"/>
-      <c r="AP4" s="11"/>
-      <c r="AQ4" s="11"/>
-      <c r="AR4" s="11"/>
+      <c r="Q4" s="15"/>
+      <c r="R4" s="15"/>
+      <c r="S4" s="15"/>
+      <c r="T4" s="15"/>
+      <c r="U4" s="15"/>
+      <c r="V4" s="15"/>
+      <c r="W4" s="15"/>
+      <c r="X4" s="15"/>
+      <c r="Y4" s="15"/>
+      <c r="Z4" s="15"/>
+      <c r="AA4" s="15"/>
+      <c r="AB4" s="15"/>
+      <c r="AC4" s="14"/>
+      <c r="AD4" s="14"/>
+      <c r="AE4" s="16"/>
+      <c r="AF4" s="7"/>
+      <c r="AG4" s="8"/>
+      <c r="AH4" s="8"/>
+      <c r="AI4" s="9"/>
+      <c r="AJ4" s="9"/>
+      <c r="AK4" s="10"/>
+      <c r="AL4" s="10"/>
+      <c r="AM4" s="10"/>
+      <c r="AN4" s="11"/>
+      <c r="AO4" s="12"/>
+      <c r="AP4" s="12"/>
+      <c r="AQ4" s="12"/>
+      <c r="AR4" s="12"/>
       <c r="AMG4" s="0"/>
       <c r="AMH4" s="0"/>
       <c r="AMI4" s="0"/>
       <c r="AMJ4" s="0"/>
     </row>
     <row r="5" customFormat="false" ht="15.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="17" t="s">
+      <c r="B5" s="5"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="L5" s="17"/>
-      <c r="M5" s="18" t="s">
+      <c r="L5" s="18"/>
+      <c r="M5" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="N5" s="18"/>
-      <c r="O5" s="19" t="s">
+      <c r="N5" s="19"/>
+      <c r="O5" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="P5" s="17" t="s">
+      <c r="P5" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="Q5" s="17"/>
-      <c r="R5" s="17"/>
-      <c r="S5" s="17"/>
-      <c r="T5" s="17"/>
-      <c r="U5" s="17" t="s">
+      <c r="Q5" s="18"/>
+      <c r="R5" s="18"/>
+      <c r="S5" s="18"/>
+      <c r="T5" s="18"/>
+      <c r="U5" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="V5" s="17"/>
-      <c r="W5" s="17"/>
-      <c r="X5" s="17"/>
-      <c r="Y5" s="17"/>
-      <c r="Z5" s="18" t="s">
+      <c r="V5" s="18"/>
+      <c r="W5" s="18"/>
+      <c r="X5" s="18"/>
+      <c r="Y5" s="18"/>
+      <c r="Z5" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="AA5" s="18"/>
-      <c r="AB5" s="18" t="s">
+      <c r="AA5" s="19"/>
+      <c r="AB5" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="AC5" s="18" t="s">
+      <c r="AC5" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="AD5" s="18"/>
-      <c r="AE5" s="18"/>
-      <c r="AF5" s="6"/>
-      <c r="AG5" s="7"/>
-      <c r="AH5" s="7"/>
-      <c r="AI5" s="8"/>
-      <c r="AJ5" s="8"/>
-      <c r="AK5" s="9"/>
-      <c r="AL5" s="9"/>
-      <c r="AM5" s="9"/>
-      <c r="AN5" s="10"/>
-      <c r="AO5" s="10"/>
-      <c r="AP5" s="11"/>
-      <c r="AQ5" s="11"/>
-      <c r="AR5" s="11"/>
+      <c r="AD5" s="19"/>
+      <c r="AE5" s="19"/>
+      <c r="AF5" s="7"/>
+      <c r="AG5" s="8"/>
+      <c r="AH5" s="8"/>
+      <c r="AI5" s="9"/>
+      <c r="AJ5" s="9"/>
+      <c r="AK5" s="10"/>
+      <c r="AL5" s="10"/>
+      <c r="AM5" s="10"/>
+      <c r="AN5" s="11"/>
+      <c r="AO5" s="11"/>
+      <c r="AP5" s="12"/>
+      <c r="AQ5" s="12"/>
+      <c r="AR5" s="12"/>
     </row>
-    <row r="6" s="20" customFormat="true" ht="72.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="20" t="s">
+    <row r="6" s="21" customFormat="true" ht="52.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="22" t="s">
         <v>52</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="C6" s="22" t="s">
         <v>53</v>
       </c>
-      <c r="D6" s="21" t="s">
+      <c r="D6" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="E6" s="21" t="s">
+      <c r="E6" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="F6" s="21" t="s">
+      <c r="F6" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="G6" s="21" t="s">
+      <c r="G6" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="H6" s="21" t="s">
+      <c r="H6" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="I6" s="21" t="s">
+      <c r="I6" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="J6" s="22" t="s">
+      <c r="J6" s="23" t="s">
         <v>60</v>
       </c>
-      <c r="K6" s="23" t="s">
+      <c r="K6" s="24" t="s">
         <v>61</v>
       </c>
-      <c r="L6" s="24" t="s">
+      <c r="L6" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="M6" s="24" t="s">
+      <c r="M6" s="25" t="s">
         <v>63</v>
       </c>
-      <c r="N6" s="24" t="s">
+      <c r="N6" s="25" t="s">
         <v>64</v>
       </c>
-      <c r="O6" s="23" t="s">
+      <c r="O6" s="24" t="s">
         <v>46</v>
       </c>
-      <c r="P6" s="24" t="s">
+      <c r="P6" s="25" t="s">
         <v>65</v>
       </c>
-      <c r="Q6" s="24" t="s">
+      <c r="Q6" s="25" t="s">
         <v>66</v>
       </c>
-      <c r="R6" s="24" t="s">
+      <c r="R6" s="25" t="s">
         <v>67</v>
       </c>
-      <c r="S6" s="24" t="s">
+      <c r="S6" s="25" t="s">
         <v>68</v>
       </c>
-      <c r="T6" s="24" t="s">
+      <c r="T6" s="25" t="s">
         <v>69</v>
       </c>
-      <c r="U6" s="24" t="s">
+      <c r="U6" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="V6" s="24" t="s">
+      <c r="V6" s="25" t="s">
         <v>71</v>
       </c>
-      <c r="W6" s="24" t="s">
+      <c r="W6" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="X6" s="24" t="s">
+      <c r="X6" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="Y6" s="24" t="s">
+      <c r="Y6" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="Z6" s="24" t="s">
+      <c r="Z6" s="25" t="s">
         <v>75</v>
       </c>
-      <c r="AA6" s="24" t="s">
+      <c r="AA6" s="25" t="s">
         <v>76</v>
       </c>
-      <c r="AB6" s="24" t="s">
+      <c r="AB6" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="AC6" s="24" t="s">
+      <c r="AC6" s="25" t="s">
         <v>78</v>
       </c>
-      <c r="AD6" s="24" t="s">
+      <c r="AD6" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="AE6" s="24" t="s">
+      <c r="AE6" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="AF6" s="25" t="s">
+      <c r="AF6" s="26" t="s">
         <v>81</v>
       </c>
-      <c r="AG6" s="26" t="s">
+      <c r="AG6" s="27" t="s">
         <v>82</v>
       </c>
-      <c r="AH6" s="26" t="s">
+      <c r="AH6" s="27" t="s">
         <v>83</v>
       </c>
-      <c r="AI6" s="26" t="s">
+      <c r="AI6" s="27" t="s">
         <v>84</v>
       </c>
-      <c r="AJ6" s="26" t="s">
+      <c r="AJ6" s="27" t="s">
         <v>85</v>
       </c>
-      <c r="AK6" s="27" t="s">
+      <c r="AK6" s="28" t="s">
         <v>86</v>
       </c>
-      <c r="AL6" s="27" t="s">
+      <c r="AL6" s="28" t="s">
         <v>87</v>
       </c>
-      <c r="AM6" s="27" t="s">
+      <c r="AM6" s="28" t="s">
         <v>88</v>
       </c>
-      <c r="AN6" s="24" t="s">
+      <c r="AN6" s="25" t="s">
         <v>89</v>
       </c>
-      <c r="AO6" s="28" t="s">
+      <c r="AO6" s="29" t="s">
         <v>90</v>
       </c>
-      <c r="AP6" s="28" t="s">
+      <c r="AP6" s="29" t="s">
         <v>91</v>
       </c>
-      <c r="AQ6" s="28" t="s">
+      <c r="AQ6" s="29" t="s">
         <v>92</v>
       </c>
-      <c r="AR6" s="29" t="s">
+      <c r="AR6" s="30" t="s">
         <v>93</v>
       </c>
       <c r="AMG6" s="0"/>
@@ -1509,85 +1524,85 @@
       <c r="AMI6" s="0"/>
       <c r="AMJ6" s="0"/>
     </row>
-    <row r="7" s="16" customFormat="true" ht="8.65" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="16" t="s">
+    <row r="7" s="17" customFormat="true" ht="17.35" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="B7" s="30" t="s">
+      <c r="B7" s="31" t="s">
         <v>94</v>
       </c>
-      <c r="C7" s="30"/>
-      <c r="D7" s="30"/>
-      <c r="E7" s="30"/>
-      <c r="F7" s="30"/>
-      <c r="G7" s="30"/>
-      <c r="H7" s="30"/>
-      <c r="I7" s="30"/>
-      <c r="J7" s="30"/>
-      <c r="K7" s="31" t="n">
+      <c r="C7" s="31"/>
+      <c r="D7" s="31"/>
+      <c r="E7" s="31"/>
+      <c r="F7" s="31"/>
+      <c r="G7" s="31"/>
+      <c r="H7" s="31"/>
+      <c r="I7" s="31"/>
+      <c r="J7" s="31"/>
+      <c r="K7" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="L7" s="31" t="n">
+      <c r="L7" s="32" t="n">
         <v>2</v>
       </c>
-      <c r="M7" s="31" t="n">
+      <c r="M7" s="32" t="n">
         <v>3</v>
       </c>
-      <c r="N7" s="31" t="n">
+      <c r="N7" s="32" t="n">
         <v>4</v>
       </c>
-      <c r="O7" s="31" t="n">
+      <c r="O7" s="32" t="n">
         <v>5</v>
       </c>
-      <c r="P7" s="31" t="s">
+      <c r="P7" s="32" t="s">
         <v>95</v>
       </c>
-      <c r="Q7" s="32" t="s">
+      <c r="Q7" s="33" t="s">
         <v>96</v>
       </c>
-      <c r="R7" s="32" t="s">
+      <c r="R7" s="33" t="s">
         <v>97</v>
       </c>
-      <c r="S7" s="32" t="s">
+      <c r="S7" s="33" t="s">
         <v>98</v>
       </c>
-      <c r="T7" s="32" t="s">
+      <c r="T7" s="33" t="s">
         <v>99</v>
       </c>
-      <c r="U7" s="32" t="s">
+      <c r="U7" s="33" t="s">
         <v>100</v>
       </c>
-      <c r="V7" s="32" t="s">
+      <c r="V7" s="33" t="s">
         <v>101</v>
       </c>
-      <c r="W7" s="32" t="s">
+      <c r="W7" s="33" t="s">
         <v>102</v>
       </c>
-      <c r="X7" s="31" t="s">
+      <c r="X7" s="32" t="s">
         <v>103</v>
       </c>
-      <c r="Y7" s="32" t="s">
+      <c r="Y7" s="33" t="s">
         <v>104</v>
       </c>
-      <c r="Z7" s="31" t="s">
+      <c r="Z7" s="32" t="s">
         <v>105</v>
       </c>
-      <c r="AA7" s="32" t="s">
+      <c r="AA7" s="33" t="s">
         <v>106</v>
       </c>
-      <c r="AB7" s="31" t="s">
+      <c r="AB7" s="32" t="s">
         <v>107</v>
       </c>
-      <c r="AC7" s="31" t="s">
+      <c r="AC7" s="32" t="s">
         <v>108</v>
       </c>
-      <c r="AD7" s="31" t="s">
+      <c r="AD7" s="32" t="s">
         <v>109</v>
       </c>
-      <c r="AE7" s="31" t="s">
+      <c r="AE7" s="32" t="s">
         <v>110</v>
       </c>
-      <c r="AF7" s="31"/>
+      <c r="AF7" s="32"/>
       <c r="AG7" s="0"/>
       <c r="AH7" s="0"/>
       <c r="AI7" s="0"/>
@@ -1647,7 +1662,7 @@
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Page &amp;P</oddFooter>
@@ -1661,7 +1676,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultColWidth="8.48828125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="0" width="11.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15.53"/>
@@ -1682,7 +1697,7 @@
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="true" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="12.65" hidden="true" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -1692,13 +1707,13 @@
       <c r="C2" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="D2" s="33" t="s">
+      <c r="D2" s="34" t="s">
         <v>113</v>
       </c>
-      <c r="E2" s="33" t="s">
+      <c r="E2" s="34" t="s">
         <v>114</v>
       </c>
-      <c r="F2" s="33" t="s">
+      <c r="F2" s="35" t="s">
         <v>115</v>
       </c>
       <c r="G2" s="2" t="s">
@@ -1712,30 +1727,30 @@
       <c r="A3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="34" t="s">
+      <c r="B3" s="36" t="s">
         <v>118</v>
       </c>
-      <c r="C3" s="34" t="s">
+      <c r="C3" s="36" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="35" t="s">
+      <c r="D3" s="37" t="s">
         <v>119</v>
       </c>
-      <c r="E3" s="35" t="s">
+      <c r="E3" s="37" t="s">
         <v>94</v>
       </c>
-      <c r="F3" s="35" t="s">
+      <c r="F3" s="37" t="s">
         <v>120</v>
       </c>
-      <c r="G3" s="34" t="s">
+      <c r="G3" s="36" t="s">
         <v>121</v>
       </c>
-      <c r="H3" s="34" t="s">
+      <c r="H3" s="36" t="s">
         <v>122</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B3:H4"/>
+  <autoFilter ref="B3:H3"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>